<commit_message>
Improve C3DC filter stability, Memgraph logging
</commit_message>
<xml_diff>
--- a/InputFiles/C3DC/TC04_C3DC_phs000467_AnatoSite-Liver.xlsx
+++ b/InputFiles/C3DC/TC04_C3DC_phs000467_AnatoSite-Liver.xlsx
@@ -509,7 +509,7 @@
         <is>
           <t>MATCH (p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
 WHERE s.dbgap_accession = 'phs000467'
-  AND EXISTS { MATCH (d:diagnosis)-[:of_diagnosis]-&gt;(p) WHERE 'C22.0 : Liver' IN coalesce(d.anatomic_site, []) }
+  AND EXISTS { MATCH (d:diagnosis)-[:of_diagnosis]-&gt;(p) WHERE 'liver' IN coalesce(d.anatomic_site, []) }
 RETURN p.participant_id AS `Participant ID`,
        s.study_id AS `Study ID`,
        p.sex_at_birth AS `Sex at Birth`,
@@ -522,7 +522,7 @@
         <is>
           <t>MATCH (p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
 WHERE s.dbgap_accession = 'phs000467'
-  AND EXISTS { MATCH (d:diagnosis)-[:of_diagnosis]-&gt;(p) WHERE 'C22.0 : Liver' IN coalesce(d.anatomic_site, []) }
+  AND EXISTS { MATCH (d:diagnosis)-[:of_diagnosis]-&gt;(p) WHERE 'liver' IN coalesce(d.anatomic_site, []) }
 OPTIONAL MATCH (sm:sample)-[:of_sample]-&gt;(p)
 OPTIONAL MATCH (f)-[:of_sequencing_file|of_clinical_measure_file|of_cytogenomic_file|of_generic_file|of_methylation_array_file|of_pathology_file|of_radiology_file]-&gt;(sm)
 OPTIONAL MATCH (fp)-[:of_clinical_measure_file|of_generic_file|of_radiology_file]-&gt;(p)
@@ -554,7 +554,7 @@
           <t>MATCH (s:study)
 WHERE EXISTS {
   MATCH (d:diagnosis)-[:of_diagnosis]-&gt;(p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s)
-  WHERE s.dbgap_accession = 'phs000467' AND 'C22.0 : Liver' IN coalesce(d.anatomic_site, [])
+  WHERE s.dbgap_accession = 'phs000467' AND 'liver' IN coalesce(d.anatomic_site, [])
 }
 WITH s
 MATCH (sp:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s)
@@ -635,7 +635,7 @@
         <is>
           <t>MATCH (d:diagnosis)-[:of_diagnosis]-&gt;(p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
 WHERE s.dbgap_accession = 'phs000467'
-  AND 'C22.0 : Liver' IN coalesce(d.anatomic_site, [])
+  AND 'liver' IN coalesce(d.anatomic_site, [])
 RETURN p.participant_id AS `Participant ID`,
        d.diagnosis_id AS `Diagnosis ID`,
        d.diagnosis AS `Diagnosis`,
@@ -661,7 +661,7 @@
         <is>
           <t>MATCH (g:genetic_analysis)-[:of_genetic_analysis]-&gt;(:sample)-[:of_sample]-&gt;(p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
 WHERE s.dbgap_accession = 'phs000467'
-  AND EXISTS { MATCH (d:diagnosis)-[:of_diagnosis]-&gt;(p) WHERE 'C22.0 : Liver' IN coalesce(d.anatomic_site, []) }
+  AND EXISTS { MATCH (d:diagnosis)-[:of_diagnosis]-&gt;(p) WHERE 'liver' IN coalesce(d.anatomic_site, []) }
 WITH p, g, s,
      CASE
        WHEN g.gene_symbol IS NULL THEN []
@@ -695,7 +695,7 @@
         <is>
           <t>CALL {
   MATCH (t:treatment_chemotherapy)-[:of_treatment_chemotherapy]-&gt;(p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
-  WHERE s.dbgap_accession = 'phs000467' AND EXISTS { MATCH (d:diagnosis)-[:of_diagnosis]-&gt;(p) WHERE 'C22.0 : Liver' IN coalesce(d.anatomic_site, []) }
+  WHERE s.dbgap_accession = 'phs000467' AND EXISTS { MATCH (d:diagnosis)-[:of_diagnosis]-&gt;(p) WHERE 'liver' IN coalesce(d.anatomic_site, []) }
   RETURN p.participant_id AS participant_id,
          t.treatment_chemotherapy_id AS treatment_id,
          CASE WHEN t.age_at_treatment_start IS NULL OR t.age_at_treatment_start = -999 THEN 'Not Reported' ELSE toString(t.age_at_treatment_start) END AS age_start,
@@ -705,7 +705,7 @@
          s.dbgap_accession AS dbgap_accession
   UNION
   MATCH (t:treatment_radiation)-[:of_treatment_radiation]-&gt;(p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
-  WHERE s.dbgap_accession = 'phs000467' AND EXISTS { MATCH (d:diagnosis)-[:of_diagnosis]-&gt;(p) WHERE 'C22.0 : Liver' IN coalesce(d.anatomic_site, []) }
+  WHERE s.dbgap_accession = 'phs000467' AND EXISTS { MATCH (d:diagnosis)-[:of_diagnosis]-&gt;(p) WHERE 'liver' IN coalesce(d.anatomic_site, []) }
   RETURN p.participant_id AS participant_id,
          t.treatment_radiation_id AS treatment_id,
          CASE WHEN t.age_at_treatment_start IS NULL OR t.age_at_treatment_start = -999 THEN 'Not Reported' ELSE toString(t.age_at_treatment_start) END AS age_start,
@@ -715,7 +715,7 @@
          s.dbgap_accession AS dbgap_accession
   UNION
   MATCH (t:treatment_surgery)-[:of_treatment_surgery]-&gt;(p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
-  WHERE s.dbgap_accession = 'phs000467' AND EXISTS { MATCH (d:diagnosis)-[:of_diagnosis]-&gt;(p) WHERE 'C22.0 : Liver' IN coalesce(d.anatomic_site, []) }
+  WHERE s.dbgap_accession = 'phs000467' AND EXISTS { MATCH (d:diagnosis)-[:of_diagnosis]-&gt;(p) WHERE 'liver' IN coalesce(d.anatomic_site, []) }
   RETURN p.participant_id AS participant_id,
          t.treatment_surgery_id AS treatment_id,
          CASE WHEN t.age_at_treatment_start IS NULL OR t.age_at_treatment_start = -999 THEN 'Not Reported' ELSE toString(t.age_at_treatment_start) END AS age_start,
@@ -725,7 +725,7 @@
          s.dbgap_accession AS dbgap_accession
   UNION
   MATCH (t:treatment_other)-[:of_treatment_other]-&gt;(p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
-  WHERE s.dbgap_accession = 'phs000467' AND EXISTS { MATCH (d:diagnosis)-[:of_diagnosis]-&gt;(p) WHERE 'C22.0 : Liver' IN coalesce(d.anatomic_site, []) }
+  WHERE s.dbgap_accession = 'phs000467' AND EXISTS { MATCH (d:diagnosis)-[:of_diagnosis]-&gt;(p) WHERE 'liver' IN coalesce(d.anatomic_site, []) }
   RETURN p.participant_id AS participant_id,
          t.treatment_other_id AS treatment_id,
          CASE WHEN t.age_at_treatment_start IS NULL OR t.age_at_treatment_start = -999 THEN 'Not Reported' ELSE toString(t.age_at_treatment_start) END AS age_start,
@@ -756,7 +756,7 @@
         <is>
           <t>MATCH (tr:treatment_response)-[:of_treatment_response]-&gt;(p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
 WHERE s.dbgap_accession = 'phs000467'
-  AND EXISTS { MATCH (d:diagnosis)-[:of_diagnosis]-&gt;(p) WHERE 'C22.0 : Liver' IN coalesce(d.anatomic_site, []) }
+  AND EXISTS { MATCH (d:diagnosis)-[:of_diagnosis]-&gt;(p) WHERE 'liver' IN coalesce(d.anatomic_site, []) }
 RETURN p.participant_id AS `Participant ID`,
        tr.treatment_response_id AS `Treatment Response ID`,
        reduce(text = '', item IN coalesce(tr.response, []) | CASE WHEN text = '' THEN item ELSE text + ', ' + item END) AS `Response`,
@@ -780,7 +780,7 @@
         <is>
           <t>MATCH (sv:survival)-[:of_survival]-&gt;(p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
 WHERE s.dbgap_accession = 'phs000467'
-  AND EXISTS { MATCH (d:diagnosis)-[:of_diagnosis]-&gt;(p) WHERE 'C22.0 : Liver' IN coalesce(d.anatomic_site, []) }
+  AND EXISTS { MATCH (d:diagnosis)-[:of_diagnosis]-&gt;(p) WHERE 'liver' IN coalesce(d.anatomic_site, []) }
 RETURN p.participant_id AS `Participant ID`,
        sv.survival_id AS `Survival ID`,
        sv.last_known_survival_status AS `Last Known Survival Status`,
@@ -804,7 +804,7 @@
         <is>
           <t xml:space="preserve">MATCH (sm:sample)-[:of_sample]-&gt;(p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
 WHERE s.dbgap_accession = 'phs000467'
-  AND EXISTS { MATCH (d:diagnosis)-[:of_diagnosis]-&gt;(p) WHERE 'C22.0 : Liver' IN coalesce(d.anatomic_site, []) }
+  AND EXISTS { MATCH (d:diagnosis)-[:of_diagnosis]-&gt;(p) WHERE 'liver' IN coalesce(d.anatomic_site, []) }
 RETURN p.participant_id AS `Participant ID`,
        sm.sample_id AS `Sample ID`,
        s.study_id AS `Study ID`,
@@ -831,7 +831,7 @@
         <is>
           <t>MATCH (p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
 WHERE s.dbgap_accession = 'phs000467'
-  AND EXISTS { MATCH (d:diagnosis)-[:of_diagnosis]-&gt;(p) WHERE 'C22.0 : Liver' IN coalesce(d.anatomic_site, []) }
+  AND EXISTS { MATCH (d:diagnosis)-[:of_diagnosis]-&gt;(p) WHERE 'liver' IN coalesce(d.anatomic_site, []) }
 MATCH (sm:sample)-[:of_sample]-&gt;(p)
 MATCH (f)-[:of_sequencing_file|of_clinical_measure_file|of_cytogenomic_file|of_generic_file|of_methylation_array_file|of_pathology_file|of_radiology_file]-&gt;(sm)
 RETURN f.file_name AS `File Name`,

</xml_diff>